<commit_message>
Educacion: laminas con formato propio, textos, glosario e informes 2024
</commit_message>
<xml_diff>
--- a/output/graficos_educacion_tasas/plot_regional_e_matricula_a_2018_antofagasta.xlsx
+++ b/output/graficos_educacion_tasas/plot_regional_e_matricula_a_2018_antofagasta.xlsx
@@ -6,27 +6,30 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Tasas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Niveles" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Metadata" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Detalle_region" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Detalle_nacional" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Por_edad" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Escala" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Detalle_nacional'!$A$1:$C$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Escala'!$A$1:$B$2</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t xml:space="preserve">Nivel</t>
   </si>
   <si>
-    <t xml:space="preserve">Tasa bruta (%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tasa neta (%)</t>
+    <t xml:space="preserve">Tasa neta región (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tasa neta país (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diferencia (pts)</t>
   </si>
   <si>
     <t xml:space="preserve">Preescolar</t>
@@ -50,7 +53,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-23 15:55</t>
+    <t xml:space="preserve">2026-09-30 04:11</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -68,64 +71,76 @@
     <t xml:space="preserve">Indicador</t>
   </si>
   <si>
-    <t xml:space="preserve"/>
+    <t xml:space="preserve">E_MATRICULA_a</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad territorial</t>
   </si>
   <si>
+    <t xml:space="preserve">Región de Antofagasta</t>
+  </si>
+  <si>
     <t xml:space="preserve">Año</t>
   </si>
   <si>
+    <t xml:space="preserve">2018</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tramo de edad</t>
   </si>
   <si>
-    <t xml:space="preserve">Valor regional (%)</t>
+    <t xml:space="preserve">Región (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">País (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 a 1 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 a 3 años</t>
   </si>
   <si>
     <t xml:space="preserve">4 a 5 años</t>
   </si>
   <si>
-    <t xml:space="preserve">2 a 3 años</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0 a 1 años</t>
+    <t xml:space="preserve">6 a 9 años</t>
   </si>
   <si>
     <t xml:space="preserve">10 a 13 años</t>
   </si>
   <si>
-    <t xml:space="preserve">6 a 9 años</t>
+    <t xml:space="preserve">14 a 15 años</t>
   </si>
   <si>
     <t xml:space="preserve">16 a 17 años</t>
   </si>
   <si>
-    <t xml:space="preserve">14 a 15 años</t>
+    <t xml:space="preserve">18 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 años</t>
   </si>
   <si>
     <t xml:space="preserve">24 años</t>
   </si>
   <si>
-    <t xml:space="preserve">23 años</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22 años</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21 años</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20 años</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19 años</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18 años</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor nacional (%)</t>
+    <t xml:space="preserve">Mínimo de la escala (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Máximo de la escala (%)</t>
   </si>
 </sst>
 </file>
@@ -491,8 +506,9 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="12.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="16.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="15.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="22.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="20.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="18.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -505,53 +521,68 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45.91</v>
+        <v>45.7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45.71</v>
+        <v>52.2</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>-6.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>97.83</v>
+        <v>93.3</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>93.27</v>
+        <v>95.1</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>-1.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>103.06</v>
+        <v>81.9</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>81.86</v>
+        <v>82.3</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>-0.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>60.97</v>
+        <v>39.3</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>39.3</v>
+        <v>41.1</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>-1.8</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C5"/>
+  <autoFilter ref="A1:D5"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
@@ -568,58 +599,58 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -635,7 +666,9 @@
   <cols>
     <col min="1" max="1" width="12.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="15.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="20.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="12.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="10.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="18.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -643,168 +676,258 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>83.42</v>
+        <v>13.3</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>-4.2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>37.85</v>
+        <v>37.9</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>13.31</v>
+        <v>83.4</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>-4.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>92.49</v>
+        <v>94</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>-2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>93.99</v>
+        <v>92.5</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>-1.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>80.93</v>
+        <v>82.8</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>82.7</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>82.81</v>
+        <v>80.9</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>-0.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>24.99</v>
+        <v>39.8</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>2.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>30.93</v>
+        <v>51.9</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>-0.3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>37.19</v>
+        <v>49.5</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>-3.3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>44.76</v>
+        <v>44.8</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>-3.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>49.49</v>
+        <v>37.2</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>-4.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="D14" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="C14" s="2" t="n">
-        <v>51.9</v>
+      <c r="E14" s="2" t="n">
+        <v>-2.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>39.84</v>
+        <v>25</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>-0.2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C15"/>
+  <autoFilter ref="A1:E15"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
@@ -815,178 +938,28 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="12.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="15.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="20.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="25.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="25.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>87.99</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>51.9</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>17.52</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>94.19</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>96.03</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>81.83</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>82.73</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>25.18</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>33.01</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>41.45</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>48.24</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>52.81</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>52.18</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>37.46</v>
+      <c r="A2" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C15"/>
+  <autoFilter ref="A1:B2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>

</xml_diff>